<commit_message>
Add SOH report for 2026-10-23
</commit_message>
<xml_diff>
--- a/reports/SOH_23_10_2026.xlsx
+++ b/reports/SOH_23_10_2026.xlsx
@@ -433,7 +433,7 @@
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="21" customWidth="1" min="2" max="2"/>
-    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="65" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
@@ -2682,7 +2682,7 @@
         </is>
       </c>
       <c r="D80" s="2" t="n">
-        <v>1315</v>
+        <v>1309</v>
       </c>
       <c r="E80" s="3" t="n">
         <v>14093</v>
@@ -3214,7 +3214,7 @@
         </is>
       </c>
       <c r="D99" s="2" t="n">
-        <v>710</v>
+        <v>704</v>
       </c>
       <c r="E99" s="3" t="n">
         <v>25495</v>
@@ -3578,7 +3578,7 @@
         </is>
       </c>
       <c r="D112" s="2" t="n">
-        <v>286</v>
+        <v>280</v>
       </c>
       <c r="E112" s="3" t="n">
         <v>14320</v>
@@ -3942,7 +3942,7 @@
         </is>
       </c>
       <c r="D125" s="2" t="n">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="E125" s="3" t="n">
         <v>13595</v>
@@ -9774,7 +9774,7 @@
         </is>
       </c>
       <c r="D337" s="2" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E337" s="3" t="n">
         <v>11171</v>
@@ -10442,7 +10442,7 @@
       </c>
       <c r="C361" t="inlineStr">
         <is>
-          <t>AIWIBI Kid's Jolly Teeth Care Toothpaste(Strawberry)</t>
+          <t>AIWIBI Kid's Jolly Teeth Care Toothpaste(Strawberry) (96*1Pc)</t>
         </is>
       </c>
       <c r="D361" s="2" t="n">
@@ -10470,7 +10470,7 @@
       </c>
       <c r="C362" t="inlineStr">
         <is>
-          <t>AIWIBI Kid's Jolly Teeth Care Toothpaste(Grape)</t>
+          <t>AIWIBI Kid's Jolly Teeth Care Toothpaste(Grape) (96*1Pc)</t>
         </is>
       </c>
       <c r="D362" s="2" t="n">
@@ -10498,7 +10498,7 @@
       </c>
       <c r="C363" t="inlineStr">
         <is>
-          <t>AIWIBI Kid's Jolly Teeth Care Toothpaste(Lemon)</t>
+          <t>AIWIBI Kid's Jolly Teeth Care Toothpaste(Lemon) (96*1Pc)</t>
         </is>
       </c>
       <c r="D363" s="2" t="n">
@@ -10526,7 +10526,7 @@
       </c>
       <c r="C364" t="inlineStr">
         <is>
-          <t>AIWIBI Kid's Jolly Teeth Care Toothpaste(Apple)</t>
+          <t>AIWIBI Kid's Jolly Teeth Care Toothpaste(Apple) (96*1Pc)</t>
         </is>
       </c>
       <c r="D364" s="2" t="n">
@@ -10554,7 +10554,7 @@
       </c>
       <c r="C365" t="inlineStr">
         <is>
-          <t>AIWIBI Kids Jolly Teeth Care (Combo)</t>
+          <t>AIWIBI Kids Jolly Teeth Care (Combo) (72*1Pc)</t>
         </is>
       </c>
       <c r="D365" s="2" t="n">
@@ -12374,7 +12374,7 @@
       </c>
       <c r="C430" t="inlineStr">
         <is>
-          <t>AWN ADULT MATERNITY PAD</t>
+          <t>AWN Adult Maternity Pad (20*12pcs)</t>
         </is>
       </c>
       <c r="D430" s="2" t="n">
@@ -15598,7 +15598,7 @@
         </is>
       </c>
       <c r="D545" s="2" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="E545" s="3" t="n">
         <v>9818</v>
@@ -23382,7 +23382,7 @@
         </is>
       </c>
       <c r="D823" s="2" t="n">
-        <v>336</v>
+        <v>325</v>
       </c>
       <c r="E823" s="3" t="n">
         <v>11606</v>
@@ -26070,7 +26070,7 @@
         </is>
       </c>
       <c r="D919" s="2" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E919" s="3" t="n">
         <v>13734</v>
@@ -26126,7 +26126,7 @@
         </is>
       </c>
       <c r="D921" s="2" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E921" s="3" t="n">
         <v>18059</v>
@@ -34247,7 +34247,7 @@
         </is>
       </c>
       <c r="D1211" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E1211" s="3" t="n">
         <v>7373</v>
@@ -34583,7 +34583,7 @@
         </is>
       </c>
       <c r="D1223" s="2" t="n">
-        <v>146</v>
+        <v>140</v>
       </c>
       <c r="E1223" s="3" t="n">
         <v>8180</v>

</xml_diff>